<commit_message>
Apply 60 percent secondee salary share
</commit_message>
<xml_diff>
--- a/projects/PetroUrdaneta-FDP9/compensation/manpower_cost_summary_single_sheet.xlsx
+++ b/projects/PetroUrdaneta-FDP9/compensation/manpower_cost_summary_single_sheet.xlsx
@@ -1257,24 +1257,24 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: management instruction in this task through 7–8 September 2026. PU pays the costs of Alexander Stulme, Alan McKeon and Martin Aguero as secondees.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>29</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>3</xdr:col>
-                <xdr:colOff>-29</xdr:colOff>
-                <xdr:row>6</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
+          <t xml:space="preserve">Source: management instruction in this task through 7–8 September 2026. Working assumption: PU reimbursement equals 60% of the relevant secondee salary only. Barbara must confirm eligibility, documentation requirements and any reimbursement cap.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>29</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>-29</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>48</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1290,24 +1290,24 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: management instruction in this task through 7–8 September 2026. PU pays the costs of Alexander Stulme, Alan McKeon and Martin Aguero as secondees.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>29</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>3</xdr:col>
-                <xdr:colOff>-29</xdr:colOff>
-                <xdr:row>6</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
+          <t xml:space="preserve">Source: management instruction in this task through 7–8 September 2026. Working assumption: PU reimbursement equals 60% of the relevant secondee salary only. Barbara must confirm eligibility, documentation requirements and any reimbursement cap.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>29</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>-29</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>48</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1323,24 +1323,24 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: management instruction in this task through 7–8 September 2026. PU pays the costs of Alexander Stulme, Alan McKeon and Martin Aguero as secondees.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>29</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>3</xdr:col>
-                <xdr:colOff>-29</xdr:colOff>
-                <xdr:row>6</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
+          <t xml:space="preserve">Source: management instruction in this task through 7–8 September 2026. Working assumption: PU reimbursement equals 60% of the relevant secondee salary only. Barbara must confirm eligibility, documentation requirements and any reimbursement cap.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>29</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>-29</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>48</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1356,24 +1356,24 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: management instruction in this task through 7–8 September 2026. PU pays the costs of Alexander Stulme, Alan McKeon and Martin Aguero as secondees.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>29</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>3</xdr:col>
-                <xdr:colOff>-29</xdr:colOff>
-                <xdr:row>6</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
+          <t xml:space="preserve">Source: management instruction in this task through 7–8 September 2026. Working assumption: PU reimbursement equals 60% of the relevant secondee salary only. Barbara must confirm eligibility, documentation requirements and any reimbursement cap.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>29</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>-29</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>48</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1389,24 +1389,24 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: management instruction in this task through 7–8 September 2026. PU pays the costs of Alexander Stulme, Alan McKeon and Martin Aguero as secondees.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>29</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>3</xdr:col>
-                <xdr:colOff>-29</xdr:colOff>
-                <xdr:row>6</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
+          <t xml:space="preserve">Source: management instruction in this task through 7–8 September 2026. Working assumption: PU reimbursement equals 60% of the relevant secondee salary only. Barbara must confirm eligibility, documentation requirements and any reimbursement cap.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>29</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>-29</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>48</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1422,24 +1422,24 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: management instruction in this task through 7–8 September 2026. PU pays the costs of Alexander Stulme, Alan McKeon and Martin Aguero as secondees.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>29</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>3</xdr:col>
-                <xdr:colOff>-29</xdr:colOff>
-                <xdr:row>6</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
+          <t xml:space="preserve">Source: management instruction in this task through 7–8 September 2026. Working assumption: PU reimbursement equals 60% of the relevant secondee salary only. Barbara must confirm eligibility, documentation requirements and any reimbursement cap.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>29</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>-29</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>48</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1455,24 +1455,24 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: management instruction in this task through 7–8 September 2026. PU pays the costs of Alexander Stulme, Alan McKeon and Martin Aguero as secondees.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>29</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>3</xdr:col>
-                <xdr:colOff>-29</xdr:colOff>
-                <xdr:row>6</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
+          <t xml:space="preserve">Source: management instruction in this task through 7–8 September 2026. Working assumption: PU reimbursement equals 60% of the relevant secondee salary only. Barbara must confirm eligibility, documentation requirements and any reimbursement cap.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>29</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>-29</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>48</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1488,24 +1488,24 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: management instruction in this task through 7–8 September 2026. PU pays the costs of Alexander Stulme, Alan McKeon and Martin Aguero as secondees.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>29</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>3</xdr:col>
-                <xdr:colOff>-29</xdr:colOff>
-                <xdr:row>6</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
+          <t xml:space="preserve">Source: management instruction in this task through 7–8 September 2026. Working assumption: PU reimbursement equals 60% of the relevant secondee salary only. Barbara must confirm eligibility, documentation requirements and any reimbursement cap.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>29</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>-29</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>48</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1521,24 +1521,24 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Source: management instruction in this task through 7–8 September 2026. PU pays the costs of Alexander Stulme, Alan McKeon and Martin Aguero as secondees.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>29</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>3</xdr:col>
-                <xdr:colOff>-29</xdr:colOff>
-                <xdr:row>6</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
+          <t xml:space="preserve">Source: management instruction in this task through 7–8 September 2026. Working assumption: PU reimbursement equals 60% of the relevant secondee salary only. Barbara must confirm eligibility, documentation requirements and any reimbursement cap.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>29</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>-29</xdr:colOff>
+                <xdr:row>7</xdr:row>
+                <xdr:rowOff>48</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -2783,7 +2783,7 @@
     <t xml:space="preserve">Blue = source input | Black = formula | Health-care cost excluded pending Airswift confirmation</t>
   </si>
   <si>
-    <t xml:space="preserve">BIG NOTE — Alexander Stulme, Alan McKeon and Martin Aguero are PU-paid secondees. Martin is already assigned to the project as a local secondee. Repatriates receive the one-time transition package in M7 and then become local. Alan remains the only expat and receives $2,000/month housing from M7.</t>
+    <t xml:space="preserve">BIG NOTE — Alexander Stulme, Alan McKeon and Martin Aguero are secondees. The model deducts an indicative 60% PU salary-share reimbursement only, pending Barbara's confirmation of eligibility and any cap. Martin is already assigned to the project as a local secondee. Repatriates receive the one-time transition package in M7 and then become local. Alan remains the only expat and receives $2,000/month housing from M7.</t>
   </si>
   <si>
     <t xml:space="preserve">OVERALL MANPOWER COST</t>
@@ -2807,13 +2807,13 @@
     <t xml:space="preserve">Year 1</t>
   </si>
   <si>
-    <t xml:space="preserve">Health care is excluded from all costs in this model. Airswift should confirm the applicable medical coverage, eligibility, insurer and price before a separate health-care cost is approved and added. For M1–M6, the eight transition roles are assumed to work 21 days on / 14 days off: 1.71 tickets per person per month, or 13.71 tickets per month in total. Ticket costs are excluded pending Airswift confirmation.</t>
+    <t xml:space="preserve">Health care is excluded from all costs in this model. Airswift should confirm the applicable medical coverage, eligibility, insurer and price before a separate health-care cost is approved and added. For M1–M6, the eight transition roles are assumed to work 21 days on / 14 days off: 1.71 tickets per person per month, or 13.71 tickets per month in total. Ticket costs are excluded pending Airswift confirmation. Barbara must confirm the 60% secondee salary-share reimbursement and any cap.</t>
   </si>
   <si>
     <t xml:space="preserve">Gross manpower cost</t>
   </si>
   <si>
-    <t xml:space="preserve">Less: PU-paid secondees</t>
+    <t xml:space="preserve">Less: PU salary share @60%</t>
   </si>
   <si>
     <t xml:space="preserve">NET manpower cost</t>
@@ -2834,7 +2834,7 @@
     <t xml:space="preserve">M7+ Basis</t>
   </si>
   <si>
-    <t xml:space="preserve">PU-Paid?</t>
+    <t xml:space="preserve">PU Salary Share</t>
   </si>
   <si>
     <t xml:space="preserve">Tickets / Mo M1–M6</t>
@@ -2873,7 +2873,7 @@
     <t xml:space="preserve">Local — Venezuela</t>
   </si>
   <si>
-    <t xml:space="preserve">No</t>
+    <t xml:space="preserve">—</t>
   </si>
   <si>
     <t xml:space="preserve">Alexander Stulme</t>
@@ -2882,7 +2882,7 @@
     <t xml:space="preserve">Drilling &amp; Well Services Manager</t>
   </si>
   <si>
-    <t xml:space="preserve">Yes</t>
+    <t xml:space="preserve">60%</t>
   </si>
   <si>
     <t xml:space="preserve">Félix Valderrama</t>
@@ -2945,7 +2945,7 @@
     <t xml:space="preserve">REFERENCES AND MODEL SCOPE</t>
   </si>
   <si>
-    <t xml:space="preserve">References: user-provided annual compensation table reviewed 7–8 September 2026, and management instructions in this task on contract type, benefits, PU secondments and cost responsibility. Health care and ticket costs are excluded pending Airswift confirmation of coverage, price and booking scope. The M1–M6 ticket plan assumes 21 days on / 14 days off and 1.71 tickets per transition role per month. This is a management-planning cost model; tax gross-up, statutory contributions, stock options and future bonus plans require separate approval and specialist review.</t>
+    <t xml:space="preserve">References: user-provided annual compensation table reviewed 7–8 September 2026, and management instructions in this task on contract type, benefits, PU secondments and cost responsibility. Health care and ticket costs are excluded pending Airswift confirmation of coverage, price and booking scope. The M1–M6 ticket plan assumes 21 days on / 14 days off and 1.71 tickets per transition role per month. Net cost reflects an indicative 60% reimbursement of relevant secondee base salaries only; Barbara must confirm the entitlement and any cap. This is a management-planning cost model; tax gross-up, statutory contributions, stock options and future bonus plans require separate approval and specialist review.</t>
   </si>
 </sst>
 </file>
@@ -3689,20 +3689,20 @@
         <v>13</v>
       </c>
       <c r="D14" s="12" t="n">
-        <f aca="false">-SUMIF($G$21:$G$29,"Yes",$L$21:$L$29)</f>
-        <v>-45000</v>
+        <f aca="false">-SUMIF($G$21:$G$29,"60%",$L$21:$L$29)*60%</f>
+        <v>-27000</v>
       </c>
       <c r="E14" s="12" t="n">
-        <f aca="false">-SUMIF($G$21:$G$29,"Yes",$M$21:$M$29)</f>
-        <v>-69500</v>
+        <f aca="false">-SUMIF($G$21:$G$29,"60%",$L$21:$L$29)*60%</f>
+        <v>-27000</v>
       </c>
       <c r="F14" s="12" t="n">
-        <f aca="false">-SUMIF($G$21:$G$29,"Yes",$N$21:$N$29)</f>
-        <v>-47000</v>
+        <f aca="false">-SUMIF($G$21:$G$29,"60%",$L$21:$L$29)*60%</f>
+        <v>-27000</v>
       </c>
       <c r="G14" s="13" t="n">
-        <f aca="false">-SUMIF($G$21:$G$29,"Yes",$O$21:$O$29)</f>
-        <v>-574500</v>
+        <f aca="false">-SUMIF($G$21:$G$29,"60%",$I$21:$I$29)*60%</f>
+        <v>-324000</v>
       </c>
       <c r="I14" s="4"/>
       <c r="J14" s="4"/>
@@ -3718,19 +3718,19 @@
       </c>
       <c r="D15" s="15" t="n">
         <f aca="false">D13+D14</f>
-        <v>69000</v>
+        <v>87000</v>
       </c>
       <c r="E15" s="15" t="n">
         <f aca="false">E13+E14</f>
-        <v>123000</v>
+        <v>165500</v>
       </c>
       <c r="F15" s="15" t="n">
         <f aca="false">F13+F14</f>
-        <v>69000</v>
+        <v>89000</v>
       </c>
       <c r="G15" s="15" t="n">
         <f aca="false">G13+G14</f>
-        <v>882000</v>
+        <v>1132500</v>
       </c>
       <c r="I15" s="4"/>
       <c r="J15" s="4"/>
@@ -4358,7 +4358,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{13F92CCC-17D2-4C4A-A5B0-C9E636234E6E}</x14:id>
+          <x14:id>{F6AC2DF3-67B1-443D-9CA8-E09E58BCBAA8}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -4375,7 +4375,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{13F92CCC-17D2-4C4A-A5B0-C9E636234E6E}">
+          <x14:cfRule type="dataBar" id="{F6AC2DF3-67B1-443D-9CA8-E09E58BCBAA8}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>

</xml_diff>